<commit_message>
Added Filter and Default
</commit_message>
<xml_diff>
--- a/order_file/Order_IO.xlsx
+++ b/order_file/Order_IO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft12474759-my.sharepoint.com/personal/etienne_desrochers_xnnov_com/Documents/Documents/GitHub/Nouveau dossier (2)/QuantumB/order_file/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="8_{71E589D0-2AD9-4317-8FC6-2B242785F678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4ACD826D-CF2B-4264-B2C4-31AAD95A06D1}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="8_{71E589D0-2AD9-4317-8FC6-2B242785F678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9964D9A-AB72-4ACB-9C74-634F534C4030}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C2DDF0E3-580A-4B29-B2E2-7B10314745D6}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="116">
   <si>
     <t>Cool_En</t>
   </si>
@@ -364,13 +364,37 @@
   </si>
   <si>
     <t>EEV-VI_En3</t>
+  </si>
+  <si>
+    <t>RESERVED1</t>
+  </si>
+  <si>
+    <t>RESERVED2</t>
+  </si>
+  <si>
+    <t>RESERVED3</t>
+  </si>
+  <si>
+    <t>RESERVED4</t>
+  </si>
+  <si>
+    <t>RESERVED5</t>
+  </si>
+  <si>
+    <t>RESERVED6</t>
+  </si>
+  <si>
+    <t>RESERVED7</t>
+  </si>
+  <si>
+    <t>RESERVED8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -392,6 +416,12 @@
     <font>
       <sz val="18"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -864,7 +894,9 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="4"/>
+      <c r="B9" s="4" t="s">
+        <v>108</v>
+      </c>
       <c r="C9" t="s">
         <v>55</v>
       </c>
@@ -1038,7 +1070,9 @@
       <c r="A25">
         <v>24</v>
       </c>
-      <c r="B25" s="3"/>
+      <c r="B25" s="4" t="s">
+        <v>109</v>
+      </c>
       <c r="C25">
         <v>1</v>
       </c>
@@ -1212,7 +1246,9 @@
       <c r="A41">
         <v>40</v>
       </c>
-      <c r="B41" s="3"/>
+      <c r="B41" s="4" t="s">
+        <v>110</v>
+      </c>
       <c r="C41">
         <v>2</v>
       </c>
@@ -1386,7 +1422,9 @@
       <c r="A57">
         <v>56</v>
       </c>
-      <c r="B57" s="3"/>
+      <c r="B57" s="4" t="s">
+        <v>111</v>
+      </c>
       <c r="C57">
         <v>3</v>
       </c>
@@ -1395,7 +1433,9 @@
       <c r="A58">
         <v>57</v>
       </c>
-      <c r="B58" s="3"/>
+      <c r="B58" s="4" t="s">
+        <v>112</v>
+      </c>
       <c r="C58" t="s">
         <v>55</v>
       </c>
@@ -1404,7 +1444,9 @@
       <c r="A59">
         <v>58</v>
       </c>
-      <c r="B59" s="3"/>
+      <c r="B59" s="4" t="s">
+        <v>113</v>
+      </c>
       <c r="C59" t="s">
         <v>55</v>
       </c>
@@ -1413,7 +1455,9 @@
       <c r="A60">
         <v>59</v>
       </c>
-      <c r="B60" s="3"/>
+      <c r="B60" s="4" t="s">
+        <v>114</v>
+      </c>
       <c r="C60" t="s">
         <v>55</v>
       </c>
@@ -1422,7 +1466,9 @@
       <c r="A61">
         <v>60</v>
       </c>
-      <c r="B61" s="3"/>
+      <c r="B61" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="C61" t="s">
         <v>55</v>
       </c>
@@ -1869,6 +1915,7 @@
       <c r="B208" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>